<commit_message>
ajoute Marpissa nivoyi femelle et mâle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82F797E9-98D7-4177-98A1-AE25EACA31CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEC1A586-EB9B-4117-9AD4-AE8BC006005A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1545" uniqueCount="893">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1547" uniqueCount="895">
   <si>
     <t>taxon</t>
   </si>
@@ -2700,6 +2700,12 @@
   </si>
   <si>
     <t>www/media/fiches/liocranum_rupicola_male.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/marpissa_nivoyi_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/marpissa_nivoyi_male.webp</t>
   </si>
 </sst>
 </file>
@@ -9480,7 +9486,13 @@
       </c>
       <c r="C491" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D491" t="s">
+        <v>893</v>
+      </c>
+      <c r="E491" t="s">
+        <v>894</v>
       </c>
     </row>
     <row r="492" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Meta menardi femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEC1A586-EB9B-4117-9AD4-AE8BC006005A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47BC08D4-6BC9-4471-ACFE-AB1138E16692}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1547" uniqueCount="895">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1548" uniqueCount="896">
   <si>
     <t>taxon</t>
   </si>
@@ -2706,6 +2706,9 @@
   </si>
   <si>
     <t>www/media/fiches/marpissa_nivoyi_male.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/meta_menardi_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -10014,7 +10017,10 @@
       </c>
       <c r="C531" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D531" t="s">
+        <v>895</v>
       </c>
     </row>
     <row r="532" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Micrommata ligurina mâle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47BC08D4-6BC9-4471-ACFE-AB1138E16692}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D861E55-79CA-4C34-A0D9-6CE8B06C378B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1548" uniqueCount="896">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1549" uniqueCount="897">
   <si>
     <t>taxon</t>
   </si>
@@ -2709,6 +2709,9 @@
   </si>
   <si>
     <t>www/media/fiches/meta_menardi_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/micrommata_ligurina_male.webp</t>
   </si>
 </sst>
 </file>
@@ -9969,7 +9972,10 @@
       </c>
       <c r="C527" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="E527" t="s">
+        <v>896</v>
       </c>
     </row>
     <row r="528" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Micrommata virescens mâle et femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D861E55-79CA-4C34-A0D9-6CE8B06C378B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9250224-4870-44D9-AB58-67E7823A281C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1549" uniqueCount="897">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1551" uniqueCount="899">
   <si>
     <t>taxon</t>
   </si>
@@ -2712,6 +2712,12 @@
   </si>
   <si>
     <t>www/media/fiches/micrommata_ligurina_male.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/micrommata_virescens_male.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/micrommata_virescens_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -9987,7 +9993,13 @@
       </c>
       <c r="C528" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D528" t="s">
+        <v>898</v>
+      </c>
+      <c r="E528" t="s">
+        <v>897</v>
       </c>
     </row>
     <row r="529" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Myrmarachne formicaria femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9250224-4870-44D9-AB58-67E7823A281C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3EF1FBC-DBBE-46D7-AB7E-6DA9926AA46F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,12 +16,11 @@
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1551" uniqueCount="899">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1552" uniqueCount="900">
   <si>
     <t>taxon</t>
   </si>
@@ -2718,6 +2717,9 @@
   </si>
   <si>
     <t>www/media/fiches/micrommata_virescens_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/myrmarachne_formicaria_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -9540,7 +9542,10 @@
       </c>
       <c r="C494" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D494" t="s">
+        <v>899</v>
       </c>
     </row>
     <row r="495" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Nigma puella femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3EF1FBC-DBBE-46D7-AB7E-6DA9926AA46F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DBB0F31-93C8-4807-912E-F5348EB64AC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1552" uniqueCount="900">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1553" uniqueCount="901">
   <si>
     <t>taxon</t>
   </si>
@@ -2720,6 +2720,9 @@
   </si>
   <si>
     <t>www/media/fiches/myrmarachne_formicaria_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/nigma_puella_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -4595,7 +4598,10 @@
       </c>
       <c r="C106" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D106" t="s">
+        <v>900</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Pachygnatha clercki femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DBB0F31-93C8-4807-912E-F5348EB64AC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2237261D-A337-4F32-830C-3329B56A8FDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1553" uniqueCount="901">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1554" uniqueCount="902">
   <si>
     <t>taxon</t>
   </si>
@@ -2723,6 +2723,9 @@
   </si>
   <si>
     <t>www/media/fiches/nigma_puella_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/pachygnatha_clercki_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -10109,7 +10112,10 @@
       </c>
       <c r="C535" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D535" t="s">
+        <v>901</v>
       </c>
     </row>
     <row r="536" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Pachygnatha listeri femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2237261D-A337-4F32-830C-3329B56A8FDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF227168-C1A5-442A-8DD3-9965EAAA4698}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1554" uniqueCount="902">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1555" uniqueCount="903">
   <si>
     <t>taxon</t>
   </si>
@@ -2726,6 +2726,9 @@
   </si>
   <si>
     <t>www/media/fiches/pachygnatha_clercki_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/pachygnatha_listeri_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -10145,7 +10148,10 @@
       </c>
       <c r="C537" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D537" t="s">
+        <v>902</v>
       </c>
     </row>
     <row r="538" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Pistius truncatus male
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF227168-C1A5-442A-8DD3-9965EAAA4698}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BB95639-E120-4896-A4E8-56FA0A381C29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,11 +16,12 @@
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1555" uniqueCount="903">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1556" uniqueCount="904">
   <si>
     <t>taxon</t>
   </si>
@@ -2729,6 +2730,9 @@
   </si>
   <si>
     <t>www/media/fiches/pachygnatha_listeri_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/pistius_truncatus_male.webp</t>
   </si>
 </sst>
 </file>
@@ -11330,7 +11334,10 @@
       </c>
       <c r="C624" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="E624" t="s">
+        <v>903</v>
       </c>
     </row>
     <row r="625" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Philaeus chrysops mâle et femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BB95639-E120-4896-A4E8-56FA0A381C29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74BD817F-9384-43BE-B89F-8F1B8CEAC3A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1556" uniqueCount="904">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1558" uniqueCount="906">
   <si>
     <t>taxon</t>
   </si>
@@ -2733,6 +2733,12 @@
   </si>
   <si>
     <t>www/media/fiches/pistius_truncatus_male.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/philaeus_chrysops_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/philaeus_chrysops_male.webp</t>
   </si>
 </sst>
 </file>
@@ -9669,7 +9675,13 @@
       </c>
       <c r="C503" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D503" t="s">
+        <v>904</v>
+      </c>
+      <c r="E503" t="s">
+        <v>905</v>
       </c>
     </row>
     <row r="504" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Philodromus margaritatus femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74BD817F-9384-43BE-B89F-8F1B8CEAC3A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{643D89C2-C19C-4A29-91BE-3729DB524B68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1558" uniqueCount="906">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1559" uniqueCount="907">
   <si>
     <t>taxon</t>
   </si>
@@ -2739,6 +2739,9 @@
   </si>
   <si>
     <t>www/media/fiches/philaeus_chrysops_male.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/philodromus_margaritatus_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -8835,7 +8838,10 @@
       </c>
       <c r="C441" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D441" t="s">
+        <v>906</v>
       </c>
     </row>
     <row r="442" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Pirata piraticus femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{643D89C2-C19C-4A29-91BE-3729DB524B68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90F3E554-307D-483C-82F6-1882D2853FBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1559" uniqueCount="907">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1560" uniqueCount="908">
   <si>
     <t>taxon</t>
   </si>
@@ -2742,6 +2742,9 @@
   </si>
   <si>
     <t>www/media/fiches/philodromus_margaritatus_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/pirata_piraticus_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -8340,7 +8343,10 @@
       </c>
       <c r="C403" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D403" t="s">
+        <v>907</v>
       </c>
     </row>
     <row r="404" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Textrix denticulata femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{166AA76D-8B17-4E91-A943-030C5E7812F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBBD2F2F-74B0-419D-B307-69DC6DD8F804}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1561" uniqueCount="909">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1562" uniqueCount="910">
   <si>
     <t>taxon</t>
   </si>
@@ -2748,6 +2748,9 @@
   </si>
   <si>
     <t>www/media/fiches/poecilochroa_variana_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/textrix_denticulata_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -3422,7 +3425,10 @@
       </c>
       <c r="C18" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D18" t="s">
+        <v>909</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Steatoda albomaculata femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBBD2F2F-74B0-419D-B307-69DC6DD8F804}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08CFEB7F-33D8-405E-B0CA-043E7BABC96E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1562" uniqueCount="910">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1563" uniqueCount="911">
   <si>
     <t>taxon</t>
   </si>
@@ -2751,6 +2751,9 @@
   </si>
   <si>
     <t>www/media/fiches/textrix_denticulata_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/steatoda_albomaculata_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -10920,7 +10923,10 @@
       </c>
       <c r="C591" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D591" t="s">
+        <v>910</v>
       </c>
     </row>
     <row r="592" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Theridiosoma gemmosum femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08CFEB7F-33D8-405E-B0CA-043E7BABC96E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3F0A3BC-5B9C-4A0B-9229-D848ABF00434}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1563" uniqueCount="911">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1564" uniqueCount="912">
   <si>
     <t>taxon</t>
   </si>
@@ -2754,6 +2754,9 @@
   </si>
   <si>
     <t>www/media/fiches/steatoda_albomaculata_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/theridiosoma_gemmosum_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -11124,7 +11127,10 @@
       </c>
       <c r="C606" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D606" t="s">
+        <v>911</v>
       </c>
     </row>
     <row r="607" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Thomisus onustus femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3F0A3BC-5B9C-4A0B-9229-D848ABF00434}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B3F961E-688C-4007-BF19-9D66E9498986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1564" uniqueCount="912">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1565" uniqueCount="913">
   <si>
     <t>taxon</t>
   </si>
@@ -2757,6 +2757,9 @@
   </si>
   <si>
     <t>www/media/fiches/theridiosoma_gemmosum_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/thomisus_onustus_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -11445,7 +11448,10 @@
       </c>
       <c r="C628" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D628" t="s">
+        <v>912</v>
       </c>
     </row>
     <row r="629" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Salticus mutabilis mâle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B3F961E-688C-4007-BF19-9D66E9498986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EB02A2F-4A33-4BBE-93A0-611AEEFE458B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,12 +16,11 @@
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1565" uniqueCount="913">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1566" uniqueCount="914">
   <si>
     <t>taxon</t>
   </si>
@@ -2760,6 +2759,9 @@
   </si>
   <si>
     <t>www/media/fiches/thomisus_onustus_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/salticus_mutabilis_male.webp</t>
   </si>
 </sst>
 </file>
@@ -9848,6 +9850,9 @@
       <c r="D512" t="s">
         <v>725</v>
       </c>
+      <c r="E512" t="s">
+        <v>913</v>
+      </c>
     </row>
     <row r="513" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A513" t="s">

</xml_diff>

<commit_message>
ajoute Xysticus ulmi male
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EB02A2F-4A33-4BBE-93A0-611AEEFE458B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFA20695-8B3B-4C89-9F0F-F30A30C7E9F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1566" uniqueCount="914">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1567" uniqueCount="915">
   <si>
     <t>taxon</t>
   </si>
@@ -2762,6 +2762,9 @@
   </si>
   <si>
     <t>www/media/fiches/salticus_mutabilis_male.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/xysticus_ulmi_male.webp</t>
   </si>
 </sst>
 </file>
@@ -11704,6 +11707,9 @@
       <c r="D646" t="s">
         <v>760</v>
       </c>
+      <c r="E646" t="s">
+        <v>914</v>
+      </c>
     </row>
     <row r="647" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A647" t="s">

</xml_diff>

<commit_message>
ajoute Amaurobius similis femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFA20695-8B3B-4C89-9F0F-F30A30C7E9F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8CCAF73-1A2A-4E70-9031-218293692B76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1567" uniqueCount="915">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1568" uniqueCount="916">
   <si>
     <t>taxon</t>
   </si>
@@ -2765,6 +2765,9 @@
   </si>
   <si>
     <t>www/media/fiches/xysticus_ulmi_male.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/amaurobius_similis_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -3499,7 +3502,10 @@
       </c>
       <c r="C22" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D22" t="s">
+        <v>915</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajout de Aculepeira ceropegia femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8CCAF73-1A2A-4E70-9031-218293692B76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68F92241-7D7D-4793-A4E3-6C03EF51F113}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1568" uniqueCount="916">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1569" uniqueCount="917">
   <si>
     <t>taxon</t>
   </si>
@@ -2768,6 +2768,9 @@
   </si>
   <si>
     <t>www/media/fiches/amaurobius_similis_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/aculepeira_ceropegia_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -3559,7 +3562,10 @@
       </c>
       <c r="C26" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D26" t="s">
+        <v>916</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Atypus affinis femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68F92241-7D7D-4793-A4E3-6C03EF51F113}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80C696FB-A4E2-4DFA-ADED-1DBC9992E1F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1569" uniqueCount="917">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1570" uniqueCount="918">
   <si>
     <t>taxon</t>
   </si>
@@ -2771,6 +2771,9 @@
   </si>
   <si>
     <t>www/media/fiches/aculepeira_ceropegia_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/atypus_affinis_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -4088,7 +4091,10 @@
       </c>
       <c r="C63" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D63" t="s">
+        <v>917</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Atypus piceus femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80C696FB-A4E2-4DFA-ADED-1DBC9992E1F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7E46A5E-F33A-476B-8517-D5942CA5A250}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1570" uniqueCount="918">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1571" uniqueCount="919">
   <si>
     <t>taxon</t>
   </si>
@@ -2774,6 +2774,9 @@
   </si>
   <si>
     <t>www/media/fiches/atypus_affinis_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/atypus_piceus_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -4106,7 +4109,10 @@
       </c>
       <c r="C64" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D64" t="s">
+        <v>918</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Cercidia prominens femelle et remplace le mâle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7E46A5E-F33A-476B-8517-D5942CA5A250}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B20A68C8-40D0-4A74-A774-0F32F1166FEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1571" uniqueCount="919">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1572" uniqueCount="920">
   <si>
     <t>taxon</t>
   </si>
@@ -2777,6 +2777,9 @@
   </si>
   <si>
     <t>www/media/fiches/atypus_piceus_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/cercidia_prominens_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -3771,6 +3774,9 @@
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
         <v>1</v>
       </c>
+      <c r="D39" t="s">
+        <v>919</v>
+      </c>
       <c r="E39" t="s">
         <v>684</v>
       </c>

</xml_diff>

<commit_message>
ajoute Cicurina cicur femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B20A68C8-40D0-4A74-A774-0F32F1166FEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D68F1BD9-81FE-446D-85E9-340C4CF32D49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1572" uniqueCount="920">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1573" uniqueCount="921">
   <si>
     <t>taxon</t>
   </si>
@@ -2777,6 +2777,9 @@
   </si>
   <si>
     <t>www/media/fiches/atypus_piceus_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/cicurina_cicur_femelle.webp</t>
   </si>
   <si>
     <t>www/media/fiches/cercidia_prominens_femelle.webp</t>
@@ -3775,7 +3778,7 @@
         <v>1</v>
       </c>
       <c r="D39" t="s">
-        <v>919</v>
+        <v>920</v>
       </c>
       <c r="E39" t="s">
         <v>684</v>
@@ -5360,7 +5363,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>152</v>
       </c>
@@ -5372,7 +5375,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>153</v>
       </c>
@@ -5381,10 +5384,13 @@
       </c>
       <c r="C162" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="D162" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="163" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>154</v>
       </c>
@@ -5396,7 +5402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>155</v>
       </c>
@@ -5408,7 +5414,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>156</v>
       </c>
@@ -5420,7 +5426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>157</v>
       </c>
@@ -5432,7 +5438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>158</v>
       </c>
@@ -5444,7 +5450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>159</v>
       </c>
@@ -5456,7 +5462,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>160</v>
       </c>
@@ -5468,7 +5474,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>161</v>
       </c>
@@ -5480,7 +5486,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>162</v>
       </c>
@@ -5492,7 +5498,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>163</v>
       </c>
@@ -5504,7 +5510,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>164</v>
       </c>
@@ -5516,7 +5522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>165</v>
       </c>
@@ -5528,7 +5534,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>166</v>
       </c>
@@ -5540,7 +5546,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>167</v>
       </c>

</xml_diff>

<commit_message>
ajoute Crustulina guttata mâle et femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D68F1BD9-81FE-446D-85E9-340C4CF32D49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9155CCE6-C110-44FA-BD5A-27031C136273}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1573" uniqueCount="921">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1575" uniqueCount="923">
   <si>
     <t>taxon</t>
   </si>
@@ -2782,7 +2782,13 @@
     <t>www/media/fiches/cicurina_cicur_femelle.webp</t>
   </si>
   <si>
+    <t>www/media/fiches/crustulina_guttata_femelle.webp</t>
+  </si>
+  <si>
     <t>www/media/fiches/cercidia_prominens_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/crustulina_guttata_male.webp</t>
   </si>
 </sst>
 </file>
@@ -3778,7 +3784,7 @@
         <v>1</v>
       </c>
       <c r="D39" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
       <c r="E39" t="s">
         <v>684</v>
@@ -10397,7 +10403,13 @@
       </c>
       <c r="C548" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D548" t="s">
+        <v>920</v>
+      </c>
+      <c r="E548" t="s">
+        <v>922</v>
       </c>
     </row>
     <row r="549" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Dysdera erythrina femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9155CCE6-C110-44FA-BD5A-27031C136273}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AADEE14-43CC-4D3C-83A9-EE3DF64B69E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1575" uniqueCount="923">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1576" uniqueCount="924">
   <si>
     <t>taxon</t>
   </si>
@@ -2777,6 +2777,9 @@
   </si>
   <si>
     <t>www/media/fiches/atypus_piceus_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/dysdera_erythrina_femelle.webp</t>
   </si>
   <si>
     <t>www/media/fiches/cicurina_cicur_femelle.webp</t>
@@ -3784,7 +3787,7 @@
         <v>1</v>
       </c>
       <c r="D39" t="s">
-        <v>921</v>
+        <v>922</v>
       </c>
       <c r="E39" t="s">
         <v>684</v>
@@ -4727,7 +4730,10 @@
       </c>
       <c r="C109" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D109" t="s">
+        <v>919</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.3">
@@ -5393,7 +5399,7 @@
         <v>1</v>
       </c>
       <c r="D162" t="s">
-        <v>919</v>
+        <v>920</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.3">
@@ -10406,10 +10412,10 @@
         <v>1</v>
       </c>
       <c r="D548" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
       <c r="E548" t="s">
-        <v>922</v>
+        <v>923</v>
       </c>
     </row>
     <row r="549" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Episinus angulatus femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AADEE14-43CC-4D3C-83A9-EE3DF64B69E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2AA93CD-30B2-4879-99F3-FA7CF9AC354E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1576" uniqueCount="924">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1577" uniqueCount="925">
   <si>
     <t>taxon</t>
   </si>
@@ -2792,6 +2792,9 @@
   </si>
   <si>
     <t>www/media/fiches/crustulina_guttata_male.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/episinus_angulatus_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -10604,7 +10607,10 @@
       </c>
       <c r="C562" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D562" t="s">
+        <v>924</v>
       </c>
     </row>
     <row r="563" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Heliophanus kochii femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2AA93CD-30B2-4879-99F3-FA7CF9AC354E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A8B764A-A7EA-4E84-BC3B-EF41A26661C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1577" uniqueCount="925">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1578" uniqueCount="926">
   <si>
     <t>taxon</t>
   </si>
@@ -2795,6 +2795,9 @@
   </si>
   <si>
     <t>www/media/fiches/episinus_angulatus_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/heliophanus_kochii_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -9515,7 +9518,10 @@
       </c>
       <c r="C485" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D485" t="s">
+        <v>925</v>
       </c>
     </row>
     <row r="486" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Kochiura aulica femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A8B764A-A7EA-4E84-BC3B-EF41A26661C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5BACCE5-0C7C-4BF9-AA4E-EC599A64557A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1578" uniqueCount="926">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1579" uniqueCount="927">
   <si>
     <t>taxon</t>
   </si>
@@ -2798,6 +2798,9 @@
   </si>
   <si>
     <t>www/media/fiches/heliophanus_kochii_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/kochiura_aulica_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -10718,7 +10721,10 @@
       </c>
       <c r="C569" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D569" t="s">
+        <v>926</v>
       </c>
     </row>
     <row r="570" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Neoscona adianta et Neriene emphana femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5BACCE5-0C7C-4BF9-AA4E-EC599A64557A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4166A705-4307-441C-9CA7-A21CA6E66A90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1579" uniqueCount="927">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1581" uniqueCount="929">
   <si>
     <t>taxon</t>
   </si>
@@ -2801,6 +2801,12 @@
   </si>
   <si>
     <t>www/media/fiches/kochiura_aulica_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/neoscona_adianta_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/neriene_emphana_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -4024,7 +4030,10 @@
       </c>
       <c r="C56" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D56" t="s">
+        <v>927</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
@@ -6824,7 +6833,10 @@
       </c>
       <c r="C275" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D275" t="s">
+        <v>928</v>
       </c>
     </row>
     <row r="276" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Olios argelasius mâle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4166A705-4307-441C-9CA7-A21CA6E66A90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87765C43-FFB9-4F01-9860-976FB32C87D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1581" uniqueCount="929">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1582" uniqueCount="930">
   <si>
     <t>taxon</t>
   </si>
@@ -2807,6 +2807,9 @@
   </si>
   <si>
     <t>www/media/fiches/neriene_emphana_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/olios_argelasius_male.webp</t>
   </si>
 </sst>
 </file>
@@ -10157,7 +10160,10 @@
       </c>
       <c r="C529" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="E529" t="s">
+        <v>929</v>
       </c>
     </row>
     <row r="530" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Oxyopes heterophthalmus femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87765C43-FFB9-4F01-9860-976FB32C87D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06B388F3-C144-414C-AA31-930F65B47513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1582" uniqueCount="930">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1583" uniqueCount="931">
   <si>
     <t>taxon</t>
   </si>
@@ -2810,6 +2810,9 @@
   </si>
   <si>
     <t>www/media/fiches/olios_argelasius_male.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/oxyopes_heterophthalmus_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -8783,7 +8786,10 @@
       </c>
       <c r="C430" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D430" t="s">
+        <v>930</v>
       </c>
     </row>
     <row r="431" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Oxyopes ramosus femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06B388F3-C144-414C-AA31-930F65B47513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6690D22-0AF3-480A-A7A1-FB811976DB52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1583" uniqueCount="931">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1584" uniqueCount="932">
   <si>
     <t>taxon</t>
   </si>
@@ -2813,6 +2813,9 @@
   </si>
   <si>
     <t>www/media/fiches/oxyopes_heterophthalmus_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/oxyopes_ramosus_femelle.xebp</t>
   </si>
 </sst>
 </file>
@@ -8828,7 +8831,10 @@
       </c>
       <c r="C433" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D433" t="s">
+        <v>931</v>
       </c>
     </row>
     <row r="434" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
corrige le lien de la photo de Oxyopes ramosus
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6690D22-0AF3-480A-A7A1-FB811976DB52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3379BD25-6EAF-40C3-9E50-E352A89220B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2815,7 +2815,7 @@
     <t>www/media/fiches/oxyopes_heterophthalmus_femelle.webp</t>
   </si>
   <si>
-    <t>www/media/fiches/oxyopes_ramosus_femelle.xebp</t>
+    <t>www/media/fiches/oxyopes_ramosus_femelle.webp</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
ajoute Porrhomma pygmaeum femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3379BD25-6EAF-40C3-9E50-E352A89220B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2B6CA45-781A-49B5-B5FA-B38EC70C575B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1584" uniqueCount="932">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1585" uniqueCount="933">
   <si>
     <t>taxon</t>
   </si>
@@ -2816,6 +2816,9 @@
   </si>
   <si>
     <t>www/media/fiches/oxyopes_ramosus_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/porrhomma_pygmaeum_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -7250,7 +7253,10 @@
       </c>
       <c r="C307" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D307" t="s">
+        <v>932</v>
       </c>
     </row>
     <row r="308" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Araneus sturmi femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2B6CA45-781A-49B5-B5FA-B38EC70C575B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62C8D710-B035-4576-B84A-24746F07EC24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1585" uniqueCount="933">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1586" uniqueCount="934">
   <si>
     <t>taxon</t>
   </si>
@@ -2819,6 +2819,9 @@
   </si>
   <si>
     <t>www/media/fiches/porrhomma_pygmaeum_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/araneus_sturmi_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -3718,7 +3721,10 @@
       </c>
       <c r="C33" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D33" t="s">
+        <v>933</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Salticus zebraneus femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62C8D710-B035-4576-B84A-24746F07EC24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9FFB1AF-4073-4725-A3AD-7C65332BB81E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1586" uniqueCount="934">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1587" uniqueCount="935">
   <si>
     <t>taxon</t>
   </si>
@@ -2491,9 +2491,6 @@
     <t>www/media/fiches/tibellus_oblongus_male.webp</t>
   </si>
   <si>
-    <t>www/media/fiches/salticus_zebraenus_male.webp</t>
-  </si>
-  <si>
     <t>www/media/fiches/tetragnatha_extensa_male.webp</t>
   </si>
   <si>
@@ -2822,6 +2819,12 @@
   </si>
   <si>
     <t>www/media/fiches/araneus_sturmi_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/salticus_zebraneus_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/salticus_zebraneus_male.webp</t>
   </si>
 </sst>
 </file>
@@ -3400,7 +3403,7 @@
         <v>1</v>
       </c>
       <c r="D10" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
@@ -3499,7 +3502,7 @@
         <v>1</v>
       </c>
       <c r="D18" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
@@ -3526,7 +3529,7 @@
         <v>1</v>
       </c>
       <c r="D20" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
@@ -3559,7 +3562,7 @@
         <v>1</v>
       </c>
       <c r="D22" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
@@ -3616,7 +3619,7 @@
         <v>1</v>
       </c>
       <c r="D26" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
@@ -3631,7 +3634,7 @@
         <v>1</v>
       </c>
       <c r="D27" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
@@ -3646,7 +3649,7 @@
         <v>1</v>
       </c>
       <c r="D28" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
@@ -3661,7 +3664,7 @@
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
@@ -3724,7 +3727,7 @@
         <v>1</v>
       </c>
       <c r="D33" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
@@ -3739,7 +3742,7 @@
         <v>1</v>
       </c>
       <c r="D34" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
@@ -3805,7 +3808,7 @@
         <v>683</v>
       </c>
       <c r="E38" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
@@ -3820,7 +3823,7 @@
         <v>1</v>
       </c>
       <c r="D39" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="E39" t="s">
         <v>684</v>
@@ -3865,7 +3868,7 @@
         <v>1</v>
       </c>
       <c r="D42" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
@@ -3907,7 +3910,7 @@
         <v>1</v>
       </c>
       <c r="D45" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
@@ -4051,7 +4054,7 @@
         <v>1</v>
       </c>
       <c r="D56" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
@@ -4151,7 +4154,7 @@
         <v>1</v>
       </c>
       <c r="D63" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.3">
@@ -4166,7 +4169,7 @@
         <v>1</v>
       </c>
       <c r="D64" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.3">
@@ -4361,7 +4364,7 @@
         <v>1</v>
       </c>
       <c r="D79" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.3">
@@ -4490,7 +4493,7 @@
         <v>1</v>
       </c>
       <c r="D89" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="E89" t="s">
         <v>771</v>
@@ -4649,7 +4652,7 @@
         <v>772</v>
       </c>
       <c r="E101" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.3">
@@ -4676,7 +4679,7 @@
         <v>1</v>
       </c>
       <c r="D103" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="E103" t="s">
         <v>773</v>
@@ -4724,7 +4727,7 @@
         <v>1</v>
       </c>
       <c r="D106" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.3">
@@ -4769,7 +4772,7 @@
         <v>1</v>
       </c>
       <c r="D109" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.3">
@@ -4862,7 +4865,7 @@
         <v>1</v>
       </c>
       <c r="D116" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.3">
@@ -5267,7 +5270,7 @@
         <v>1</v>
       </c>
       <c r="D149" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.3">
@@ -5282,7 +5285,7 @@
         <v>1</v>
       </c>
       <c r="D150" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="E150" t="s">
         <v>776</v>
@@ -5312,7 +5315,7 @@
         <v>1</v>
       </c>
       <c r="D152" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.3">
@@ -5435,7 +5438,7 @@
         <v>1</v>
       </c>
       <c r="D162" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.3">
@@ -6218,7 +6221,7 @@
         <v>1</v>
       </c>
       <c r="D225" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
     </row>
     <row r="226" spans="1:5" x14ac:dyDescent="0.3">
@@ -6839,7 +6842,7 @@
         <v>1</v>
       </c>
       <c r="D274" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
     </row>
     <row r="275" spans="1:5" x14ac:dyDescent="0.3">
@@ -6854,7 +6857,7 @@
         <v>1</v>
       </c>
       <c r="D275" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
     </row>
     <row r="276" spans="1:5" x14ac:dyDescent="0.3">
@@ -6893,7 +6896,7 @@
         <v>1</v>
       </c>
       <c r="D278" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="E278" t="s">
         <v>675</v>
@@ -7235,7 +7238,7 @@
         <v>1</v>
       </c>
       <c r="D305" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
     </row>
     <row r="306" spans="1:4" x14ac:dyDescent="0.3">
@@ -7262,7 +7265,7 @@
         <v>1</v>
       </c>
       <c r="D307" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
     </row>
     <row r="308" spans="1:4" x14ac:dyDescent="0.3">
@@ -8018,7 +8021,7 @@
         <v>1</v>
       </c>
       <c r="E369" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
     </row>
     <row r="370" spans="1:5" x14ac:dyDescent="0.3">
@@ -8069,7 +8072,7 @@
         <v>1</v>
       </c>
       <c r="E373" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
     </row>
     <row r="374" spans="1:5" x14ac:dyDescent="0.3">
@@ -8084,7 +8087,7 @@
         <v>1</v>
       </c>
       <c r="D374" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
     </row>
     <row r="375" spans="1:5" x14ac:dyDescent="0.3">
@@ -8195,7 +8198,7 @@
         <v>1</v>
       </c>
       <c r="D383" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
     </row>
     <row r="384" spans="1:5" x14ac:dyDescent="0.3">
@@ -8237,7 +8240,7 @@
         <v>1</v>
       </c>
       <c r="E386" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
     </row>
     <row r="387" spans="1:5" x14ac:dyDescent="0.3">
@@ -8252,7 +8255,7 @@
         <v>1</v>
       </c>
       <c r="D387" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
     </row>
     <row r="388" spans="1:5" x14ac:dyDescent="0.3">
@@ -8267,7 +8270,7 @@
         <v>1</v>
       </c>
       <c r="D388" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="389" spans="1:5" x14ac:dyDescent="0.3">
@@ -8318,7 +8321,7 @@
         <v>1</v>
       </c>
       <c r="D392" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="E392" t="s">
         <v>796</v>
@@ -8396,7 +8399,7 @@
         <v>1</v>
       </c>
       <c r="E398" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
     </row>
     <row r="399" spans="1:5" x14ac:dyDescent="0.3">
@@ -8435,7 +8438,7 @@
         <v>1</v>
       </c>
       <c r="E401" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
     </row>
     <row r="402" spans="1:5" x14ac:dyDescent="0.3">
@@ -8462,7 +8465,7 @@
         <v>1</v>
       </c>
       <c r="D403" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
     </row>
     <row r="404" spans="1:5" x14ac:dyDescent="0.3">
@@ -8477,7 +8480,7 @@
         <v>1</v>
       </c>
       <c r="D404" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
     </row>
     <row r="405" spans="1:5" x14ac:dyDescent="0.3">
@@ -8702,7 +8705,7 @@
         <v>1</v>
       </c>
       <c r="D422" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
     </row>
     <row r="423" spans="1:4" x14ac:dyDescent="0.3">
@@ -8804,7 +8807,7 @@
         <v>1</v>
       </c>
       <c r="D430" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
     </row>
     <row r="431" spans="1:4" x14ac:dyDescent="0.3">
@@ -8819,7 +8822,7 @@
         <v>1</v>
       </c>
       <c r="D431" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
     </row>
     <row r="432" spans="1:4" x14ac:dyDescent="0.3">
@@ -8846,7 +8849,7 @@
         <v>1</v>
       </c>
       <c r="D433" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
     </row>
     <row r="434" spans="1:5" x14ac:dyDescent="0.3">
@@ -8882,7 +8885,7 @@
         <v>801</v>
       </c>
       <c r="E435" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
     </row>
     <row r="436" spans="1:5" x14ac:dyDescent="0.3">
@@ -8969,7 +8972,7 @@
         <v>1</v>
       </c>
       <c r="D441" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
     </row>
     <row r="442" spans="1:5" x14ac:dyDescent="0.3">
@@ -9023,7 +9026,7 @@
         <v>1</v>
       </c>
       <c r="D445" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
     </row>
     <row r="446" spans="1:5" x14ac:dyDescent="0.3">
@@ -9194,7 +9197,7 @@
         <v>1</v>
       </c>
       <c r="D458" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="E458" t="s">
         <v>705</v>
@@ -9290,7 +9293,7 @@
         <v>1</v>
       </c>
       <c r="D465" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
     </row>
     <row r="466" spans="1:5" x14ac:dyDescent="0.3">
@@ -9383,7 +9386,7 @@
         <v>1</v>
       </c>
       <c r="D472" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
     </row>
     <row r="473" spans="1:5" x14ac:dyDescent="0.3">
@@ -9458,7 +9461,7 @@
         <v>715</v>
       </c>
       <c r="E477" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
     </row>
     <row r="478" spans="1:5" x14ac:dyDescent="0.3">
@@ -9563,7 +9566,7 @@
         <v>1</v>
       </c>
       <c r="D485" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
     </row>
     <row r="486" spans="1:5" x14ac:dyDescent="0.3">
@@ -9662,10 +9665,10 @@
         <v>1</v>
       </c>
       <c r="D491" t="s">
+        <v>892</v>
+      </c>
+      <c r="E491" t="s">
         <v>893</v>
-      </c>
-      <c r="E491" t="s">
-        <v>894</v>
       </c>
     </row>
     <row r="492" spans="1:5" x14ac:dyDescent="0.3">
@@ -9704,7 +9707,7 @@
         <v>1</v>
       </c>
       <c r="D494" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
     </row>
     <row r="495" spans="1:5" x14ac:dyDescent="0.3">
@@ -9815,10 +9818,10 @@
         <v>1</v>
       </c>
       <c r="D503" t="s">
+        <v>903</v>
+      </c>
+      <c r="E503" t="s">
         <v>904</v>
-      </c>
-      <c r="E503" t="s">
-        <v>905</v>
       </c>
     </row>
     <row r="504" spans="1:5" x14ac:dyDescent="0.3">
@@ -9863,7 +9866,7 @@
         <v>804</v>
       </c>
       <c r="E506" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
     </row>
     <row r="507" spans="1:5" x14ac:dyDescent="0.3">
@@ -9881,7 +9884,7 @@
         <v>805</v>
       </c>
       <c r="E507" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
     </row>
     <row r="508" spans="1:5" x14ac:dyDescent="0.3">
@@ -9953,7 +9956,7 @@
         <v>725</v>
       </c>
       <c r="E512" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
     </row>
     <row r="513" spans="1:5" x14ac:dyDescent="0.3">
@@ -9968,7 +9971,7 @@
         <v>1</v>
       </c>
       <c r="D513" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="E513" t="s">
         <v>731</v>
@@ -9985,8 +9988,11 @@
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
         <v>1</v>
       </c>
+      <c r="D514" t="s">
+        <v>933</v>
+      </c>
       <c r="E514" t="s">
-        <v>823</v>
+        <v>934</v>
       </c>
     </row>
     <row r="515" spans="1:5" x14ac:dyDescent="0.3">
@@ -10154,7 +10160,7 @@
         <v>1</v>
       </c>
       <c r="E527" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="528" spans="1:5" x14ac:dyDescent="0.3">
@@ -10169,10 +10175,10 @@
         <v>1</v>
       </c>
       <c r="D528" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="E528" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="529" spans="1:5" x14ac:dyDescent="0.3">
@@ -10187,7 +10193,7 @@
         <v>1</v>
       </c>
       <c r="E529" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
     </row>
     <row r="530" spans="1:5" x14ac:dyDescent="0.3">
@@ -10214,7 +10220,7 @@
         <v>1</v>
       </c>
       <c r="D531" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
     </row>
     <row r="532" spans="1:5" x14ac:dyDescent="0.3">
@@ -10277,7 +10283,7 @@
         <v>1</v>
       </c>
       <c r="D535" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
     </row>
     <row r="536" spans="1:5" x14ac:dyDescent="0.3">
@@ -10292,7 +10298,7 @@
         <v>1</v>
       </c>
       <c r="D536" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="E536" t="s">
         <v>736</v>
@@ -10310,7 +10316,7 @@
         <v>1</v>
       </c>
       <c r="D537" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
     </row>
     <row r="538" spans="1:5" x14ac:dyDescent="0.3">
@@ -10343,7 +10349,7 @@
         <v>807</v>
       </c>
       <c r="E539" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
     </row>
     <row r="540" spans="1:5" x14ac:dyDescent="0.3">
@@ -10361,7 +10367,7 @@
         <v>808</v>
       </c>
       <c r="E540" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="541" spans="1:5" x14ac:dyDescent="0.3">
@@ -10376,7 +10382,7 @@
         <v>1</v>
       </c>
       <c r="D541" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="542" spans="1:5" x14ac:dyDescent="0.3">
@@ -10451,7 +10457,7 @@
         <v>1</v>
       </c>
       <c r="E547" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
     </row>
     <row r="548" spans="1:5" x14ac:dyDescent="0.3">
@@ -10466,10 +10472,10 @@
         <v>1</v>
       </c>
       <c r="D548" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="E548" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
     </row>
     <row r="549" spans="1:5" x14ac:dyDescent="0.3">
@@ -10586,10 +10592,10 @@
         <v>1</v>
       </c>
       <c r="D557" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="E557" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
     </row>
     <row r="558" spans="1:5" x14ac:dyDescent="0.3">
@@ -10604,7 +10610,7 @@
         <v>1</v>
       </c>
       <c r="E558" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
     </row>
     <row r="559" spans="1:5" x14ac:dyDescent="0.3">
@@ -10622,7 +10628,7 @@
         <v>810</v>
       </c>
       <c r="E559" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
     </row>
     <row r="560" spans="1:5" x14ac:dyDescent="0.3">
@@ -10661,7 +10667,7 @@
         <v>1</v>
       </c>
       <c r="D562" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
     </row>
     <row r="563" spans="1:5" x14ac:dyDescent="0.3">
@@ -10751,7 +10757,7 @@
         <v>811</v>
       </c>
       <c r="E568" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
     </row>
     <row r="569" spans="1:5" x14ac:dyDescent="0.3">
@@ -10766,7 +10772,7 @@
         <v>1</v>
       </c>
       <c r="D569" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
     </row>
     <row r="570" spans="1:5" x14ac:dyDescent="0.3">
@@ -11027,7 +11033,7 @@
         <v>813</v>
       </c>
       <c r="E589" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
     </row>
     <row r="590" spans="1:5" x14ac:dyDescent="0.3">
@@ -11054,7 +11060,7 @@
         <v>1</v>
       </c>
       <c r="D591" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
     </row>
     <row r="592" spans="1:5" x14ac:dyDescent="0.3">
@@ -11129,7 +11135,7 @@
         <v>1</v>
       </c>
       <c r="D596" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
     </row>
     <row r="597" spans="1:5" x14ac:dyDescent="0.3">
@@ -11204,7 +11210,7 @@
         <v>1</v>
       </c>
       <c r="E602" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
     </row>
     <row r="603" spans="1:5" x14ac:dyDescent="0.3">
@@ -11255,7 +11261,7 @@
         <v>1</v>
       </c>
       <c r="D606" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
     </row>
     <row r="607" spans="1:5" x14ac:dyDescent="0.3">
@@ -11354,7 +11360,7 @@
         <v>1</v>
       </c>
       <c r="D613" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
     </row>
     <row r="614" spans="1:5" x14ac:dyDescent="0.3">
@@ -11423,7 +11429,7 @@
         <v>1</v>
       </c>
       <c r="E618" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
     </row>
     <row r="619" spans="1:5" x14ac:dyDescent="0.3">
@@ -11441,7 +11447,7 @@
         <v>814</v>
       </c>
       <c r="E619" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
     </row>
     <row r="620" spans="1:5" x14ac:dyDescent="0.3">
@@ -11468,7 +11474,7 @@
         <v>1</v>
       </c>
       <c r="E621" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="622" spans="1:5" x14ac:dyDescent="0.3">
@@ -11495,7 +11501,7 @@
         <v>1</v>
       </c>
       <c r="E623" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
     </row>
     <row r="624" spans="1:5" x14ac:dyDescent="0.3">
@@ -11510,7 +11516,7 @@
         <v>1</v>
       </c>
       <c r="E624" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
     </row>
     <row r="625" spans="1:5" x14ac:dyDescent="0.3">
@@ -11537,7 +11543,7 @@
         <v>1</v>
       </c>
       <c r="D626" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="E626" t="s">
         <v>755</v>
@@ -11558,7 +11564,7 @@
         <v>759</v>
       </c>
       <c r="E627" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
     </row>
     <row r="628" spans="1:5" x14ac:dyDescent="0.3">
@@ -11573,7 +11579,7 @@
         <v>1</v>
       </c>
       <c r="D628" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
     </row>
     <row r="629" spans="1:5" x14ac:dyDescent="0.3">
@@ -11588,7 +11594,7 @@
         <v>1</v>
       </c>
       <c r="E629" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
     </row>
     <row r="630" spans="1:5" x14ac:dyDescent="0.3">
@@ -11618,7 +11624,7 @@
         <v>815</v>
       </c>
       <c r="E631" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
     </row>
     <row r="632" spans="1:5" x14ac:dyDescent="0.3">
@@ -11720,7 +11726,7 @@
         <v>1</v>
       </c>
       <c r="E639" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
     </row>
     <row r="640" spans="1:5" x14ac:dyDescent="0.3">
@@ -11738,7 +11744,7 @@
         <v>817</v>
       </c>
       <c r="E640" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
     </row>
     <row r="641" spans="1:5" x14ac:dyDescent="0.3">
@@ -11780,7 +11786,7 @@
         <v>1</v>
       </c>
       <c r="E643" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
     </row>
     <row r="644" spans="1:5" x14ac:dyDescent="0.3">
@@ -11822,7 +11828,7 @@
         <v>760</v>
       </c>
       <c r="E646" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
     </row>
     <row r="647" spans="1:5" x14ac:dyDescent="0.3">
@@ -11924,10 +11930,10 @@
         <v>1</v>
       </c>
       <c r="D654" t="s">
+        <v>838</v>
+      </c>
+      <c r="E654" t="s">
         <v>839</v>
-      </c>
-      <c r="E654" t="s">
-        <v>840</v>
       </c>
     </row>
     <row r="655" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Theridion varians femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9FFB1AF-4073-4725-A3AD-7C65332BB81E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D2AFC21-5582-46EB-887F-C3F185F11F1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1587" uniqueCount="935">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1588" uniqueCount="936">
   <si>
     <t>taxon</t>
   </si>
@@ -2825,6 +2825,9 @@
   </si>
   <si>
     <t>www/media/fiches/salticus_zebraneus_male.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/theridion_varians_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -11246,7 +11249,10 @@
       </c>
       <c r="C605" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D605" t="s">
+        <v>935</v>
       </c>
     </row>
     <row r="606" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Cyclosa conica mâle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D2AFC21-5582-46EB-887F-C3F185F11F1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED064EE0-6103-42E3-A9C8-5A41E70B051F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1588" uniqueCount="936">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1589" uniqueCount="937">
   <si>
     <t>taxon</t>
   </si>
@@ -2828,6 +2828,9 @@
   </si>
   <si>
     <t>www/media/fiches/theridion_varians_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/cyclosa_conica_male.webp</t>
   </si>
 </sst>
 </file>
@@ -3846,6 +3849,9 @@
       <c r="D40" t="s">
         <v>685</v>
       </c>
+      <c r="E40" t="s">
+        <v>936</v>
+      </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">

</xml_diff>

<commit_message>
ajoute Oonops domesticus male
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED064EE0-6103-42E3-A9C8-5A41E70B051F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DB3ABAC-DF59-417E-BD39-094C7BA00F84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1589" uniqueCount="937">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1590" uniqueCount="938">
   <si>
     <t>taxon</t>
   </si>
@@ -2831,6 +2831,9 @@
   </si>
   <si>
     <t>www/media/fiches/cyclosa_conica_male.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/oonops_domesticus_male.webp</t>
   </si>
 </sst>
 </file>
@@ -8639,7 +8642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="417" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="417" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A417" t="s">
         <v>386</v>
       </c>
@@ -8654,7 +8657,7 @@
         <v>798</v>
       </c>
     </row>
-    <row r="418" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="418" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A418" t="s">
         <v>387</v>
       </c>
@@ -8666,7 +8669,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="419" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="419" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A419" t="s">
         <v>388</v>
       </c>
@@ -8678,7 +8681,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="420" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="420" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A420" t="s">
         <v>389</v>
       </c>
@@ -8690,7 +8693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="421" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="421" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A421" t="s">
         <v>390</v>
       </c>
@@ -8702,7 +8705,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="422" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="422" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A422" t="s">
         <v>391</v>
       </c>
@@ -8717,7 +8720,7 @@
         <v>854</v>
       </c>
     </row>
-    <row r="423" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="423" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A423" t="s">
         <v>392</v>
       </c>
@@ -8729,7 +8732,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="424" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="424" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A424" t="s">
         <v>393</v>
       </c>
@@ -8741,7 +8744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="425" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="425" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A425" t="s">
         <v>646</v>
       </c>
@@ -8753,7 +8756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="426" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="426" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A426" t="s">
         <v>394</v>
       </c>
@@ -8767,8 +8770,11 @@
       <c r="D426" t="s">
         <v>799</v>
       </c>
-    </row>
-    <row r="427" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E426" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="427" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A427" t="s">
         <v>395</v>
       </c>
@@ -8780,7 +8786,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="428" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="428" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A428" t="s">
         <v>396</v>
       </c>
@@ -8792,7 +8798,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="429" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="429" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A429" t="s">
         <v>397</v>
       </c>
@@ -8804,7 +8810,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="430" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="430" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A430" t="s">
         <v>647</v>
       </c>
@@ -8819,7 +8825,7 @@
         <v>929</v>
       </c>
     </row>
-    <row r="431" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="431" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A431" t="s">
         <v>398</v>
       </c>
@@ -8834,7 +8840,7 @@
         <v>859</v>
       </c>
     </row>
-    <row r="432" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="432" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A432" t="s">
         <v>399</v>
       </c>

</xml_diff>

<commit_message>
ajoute Tetragnatha obtusa mâle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DB3ABAC-DF59-417E-BD39-094C7BA00F84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{153575E6-E57C-4C2B-852D-B7EBCD5E9656}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1590" uniqueCount="938">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1591" uniqueCount="939">
   <si>
     <t>taxon</t>
   </si>
@@ -2834,6 +2834,9 @@
   </si>
   <si>
     <t>www/media/fiches/oonops_domesticus_male.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/tetragnatha_obtusa_male.webp</t>
   </si>
 </sst>
 </file>
@@ -10409,7 +10412,10 @@
       </c>
       <c r="C542" t="b">
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="E542" t="s">
+        <v>938</v>
       </c>
     </row>
     <row r="543" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
ajoute Ballus chalybeius femelle
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{153575E6-E57C-4C2B-852D-B7EBCD5E9656}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A078F2CC-947F-47A8-9C0E-E4F72EDA0CD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1591" uniqueCount="939">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1592" uniqueCount="940">
   <si>
     <t>taxon</t>
   </si>
@@ -2837,6 +2837,9 @@
   </si>
   <si>
     <t>www/media/fiches/tetragnatha_obtusa_male.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/ballus_chalybeius_femelle.webp</t>
   </si>
 </sst>
 </file>
@@ -9388,6 +9391,9 @@
         <f>OR(Tableau1[[#This Row],[femelle]]&lt;&gt;"", Tableau1[[#This Row],[male]]&lt;&gt;"")</f>
         <v>1</v>
       </c>
+      <c r="D471" t="s">
+        <v>939</v>
+      </c>
       <c r="E471" t="s">
         <v>708</v>
       </c>

</xml_diff>

<commit_message>
ajoute Civizelotes civicus male
</commit_message>
<xml_diff>
--- a/photos.xlsx
+++ b/photos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\Documents\web\araignees_idf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A078F2CC-947F-47A8-9C0E-E4F72EDA0CD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{848937A7-E66A-4E16-A932-12D51223513F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1592" uniqueCount="940">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1593" uniqueCount="941">
   <si>
     <t>taxon</t>
   </si>
@@ -2840,6 +2840,9 @@
   </si>
   <si>
     <t>www/media/fiches/ballus_chalybeius_femelle.webp</t>
+  </si>
+  <si>
+    <t>www/media/fiches/civizelotes_civicus_male.webp</t>
   </si>
 </sst>
 </file>
@@ -4885,6 +4888,9 @@
       <c r="D116" t="s">
         <v>850</v>
       </c>
+      <c r="E116" t="s">
+        <v>940</v>
+      </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A117" t="s">

</xml_diff>